<commit_message>
Many more changes in files and mappings accruals
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/AQ.ST.xlsx
+++ b/data/stx_xlsx/AQ.ST.xlsx
@@ -12503,14 +12503,35 @@
       <c r="O61" s="15">
         <v>209.3</v>
       </c>
-      <c r="P61" s="19"/>
-      <c r="Q61" s="19"/>
-      <c r="R61" s="19"/>
-      <c r="S61" s="19"/>
-      <c r="T61" s="19"/>
-      <c r="U61" s="19"/>
-      <c r="V61" s="19"/>
-      <c r="W61" s="19"/>
+      <c r="P61" s="18">
+        <f t="shared" ref="P61:Q61" si="1">SUM(P62,P65,P69,P73,P86)</f>
+        <v>183.59</v>
+      </c>
+      <c r="Q61" s="18">
+        <f t="shared" si="1"/>
+        <v>185.92</v>
+      </c>
+      <c r="R61" s="18"/>
+      <c r="S61" s="18">
+        <f t="shared" ref="S61:W61" si="2">SUM(S62,S65,S69,S73,S86)</f>
+        <v>135.21</v>
+      </c>
+      <c r="T61" s="18">
+        <f t="shared" si="2"/>
+        <v>113.19</v>
+      </c>
+      <c r="U61" s="18">
+        <f t="shared" si="2"/>
+        <v>101.14</v>
+      </c>
+      <c r="V61" s="18">
+        <f t="shared" si="2"/>
+        <v>76.54</v>
+      </c>
+      <c r="W61" s="18">
+        <f t="shared" si="2"/>
+        <v>90.61</v>
+      </c>
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="14" t="s">

</xml_diff>